<commit_message>
Update Cowork-Data/multi-platform-social-post/handle-database.xlsx after Topic 3
</commit_message>
<xml_diff>
--- a/Cowork-Data/multi-platform-social-post/handle-database.xlsx
+++ b/Cowork-Data/multi-platform-social-post/handle-database.xlsx
@@ -2228,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1233"/>
+  <dimension ref="A1:Y1263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63549,6 +63549,366 @@
         </is>
       </c>
     </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>Caroline Goyder</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>Olivia Fox Cabane</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>Belle Linda Halpern</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>Diane Craig</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>Kristi Hedges</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>Carol Kinsey Goman</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>Muriel Maignan Wilkins</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>Lauren Sergy</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>Beverly Howard</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>Michael Gervais</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>Tasha Eurich</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>Victoria Labalme</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>Scott Edinger</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>Susan David</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>Tara Mohr</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>Vernice Armour</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>Peter Guber</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>John Neffinger</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>Vanessa Patrick</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>Ron Heifetz</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>Roberta Matuson</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>Jim Collins</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>Connson Locke</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>Joseph Grenny</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>Heidi Grant</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>Les Brown</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>Tom Bilyeu</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>Dan Pink</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>Patrice Washington</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>Chris Do</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -64928,7 +65288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H531"/>
+  <dimension ref="A1:H539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -84485,6 +84845,262 @@
         </is>
       </c>
     </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>69c582da20f76613b72d1500</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>2026-04-11T00:02:00Z</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>69c582db7c3be86dbd85948d</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>2026-04-11T08:02:00Z</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>69c582f420f76613b72d1572</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>2026-04-10T19:02:00Z</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F534" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>69c582f57c3be86dbd8594e5</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>2026-04-11T02:02:00Z</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>69c582f620f76613b72d1598</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>2026-04-11T04:02:00Z</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>69c582f720f76613b72d15be</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>2026-04-11T03:02:00Z</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F537" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>69c583027c3be86dbd85950b</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>2026-04-21T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="F538" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>69c583067c3be86dbd859531</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>2026-05-04T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Cowork-Data/multi-platform-social-post/handle-database.xlsx after Topic 4 - all 4 topics complete
</commit_message>
<xml_diff>
--- a/Cowork-Data/multi-platform-social-post/handle-database.xlsx
+++ b/Cowork-Data/multi-platform-social-post/handle-database.xlsx
@@ -2228,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1263"/>
+  <dimension ref="A1:Y1300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63909,6 +63909,450 @@
         </is>
       </c>
     </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>Aaron De Smet</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>Carol Dweck</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>Ray Dalio</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>Reed Hastings</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>Jez Humble</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>Jurgen Appelo</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>Mike Cottmeyer</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>Karen Martin</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>Mike Rother</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>David Marquet</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>Frederic Laloux</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>David Snowden</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>Tim Ferriss</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>Cal Newport</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>James Clear</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>Eric Ries</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>Steve Blank</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>Naval Ravikant</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>David Goggins</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>Stanley McChrystal</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>Gary Hamel</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>Charlene Li</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>Margaret Heffernan</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>Darrell Rigby</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>George Westerman</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>Tamara Erickson</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>Jeff Bezos</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>Henrik Kniberg</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>Marty Cagan</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>Gene Kim</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Jeff Sutherland</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>Simon Wardley</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Nicole Forsgren</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Marc Benioff</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Sundar Pichai</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Dean Leffingwell</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Martin Fowler</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Y1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -65288,7 +65732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H539"/>
+  <dimension ref="A1:H547"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -85101,6 +85545,262 @@
         </is>
       </c>
     </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>69c584c520f76613b72d20df</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>2026-04-11T01:01:00Z</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>69c584c77c3be86dbd859f1f</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>2026-04-11T09:01:00Z</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>69c584de20f76613b72d21c0</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>2026-04-10T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F542" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>69c584df7c3be86dbd859f79</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>2026-04-11T03:01:00Z</t>
+        </is>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>69c584e020f76613b72d21e6</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>2026-04-11T05:01:00Z</t>
+        </is>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>69c584e17c3be86dbd859f9f</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>2026-04-11T03:45:00Z</t>
+        </is>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="F545" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>69c584ec7c3be86dbd859fea</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>2026-04-28T02:00:00Z</t>
+        </is>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="F546" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>69c584f07c3be86dbd85a010</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>2026-05-11T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database: Difficult Conversations complete (Topic 3/4)
</commit_message>
<xml_diff>
--- a/Cowork-Data/multi-platform-social-post/handle-database.xlsx
+++ b/Cowork-Data/multi-platform-social-post/handle-database.xlsx
@@ -2127,7 +2127,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2147,7 +2152,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2167,7 +2177,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2187,7 +2202,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2207,7 +2222,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2228,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1300"/>
+  <dimension ref="A1:Y1249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63060,36 +63075,66 @@
     <row r="1193">
       <c r="A1193" t="inlineStr">
         <is>
-          <t>Allan Cohen</t>
+          <t>Bob Burg</t>
         </is>
       </c>
       <c r="B1193" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Burg Communications</t>
+        </is>
+      </c>
+      <c r="D1193" t="inlineStr">
+        <is>
+          <t>The Go-Giver series, influence through value</t>
         </is>
       </c>
     </row>
     <row r="1194">
       <c r="A1194" t="inlineStr">
         <is>
-          <t>David Bradford</t>
+          <t>Chris Voss</t>
         </is>
       </c>
       <c r="B1194" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>CEO &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>The Black Swan Group</t>
+        </is>
+      </c>
+      <c r="D1194" t="inlineStr">
+        <is>
+          <t>FBI negotiator, Never Split the Difference</t>
         </is>
       </c>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
         <is>
-          <t>Bob Burg</t>
+          <t>Dorie Clark</t>
         </is>
       </c>
       <c r="B1195" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Author &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D1195" t="inlineStr">
+        <is>
+          <t>Stand Out, The Long Game, building influence</t>
         </is>
       </c>
     </row>
@@ -63101,7 +63146,17 @@
       </c>
       <c r="B1196" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Yale School of Management</t>
+        </is>
+      </c>
+      <c r="D1196" t="inlineStr">
+        <is>
+          <t>Influence Is Your Superpower</t>
         </is>
       </c>
     </row>
@@ -63113,1243 +63168,2410 @@
       </c>
       <c r="B1197" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Wharton School</t>
+        </is>
+      </c>
+      <c r="D1197" t="inlineStr">
+        <is>
+          <t>The Catalyst, invisible influence</t>
         </is>
       </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
         <is>
-          <t>Chris Voss</t>
+          <t>Vanessa Bohns</t>
         </is>
       </c>
       <c r="B1198" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Cornell University</t>
+        </is>
+      </c>
+      <c r="D1198" t="inlineStr">
+        <is>
+          <t>You Have More Influence Than You Think</t>
         </is>
       </c>
     </row>
     <row r="1199">
       <c r="A1199" t="inlineStr">
         <is>
-          <t>Dorie Clark</t>
+          <t>Allan Cohen</t>
         </is>
       </c>
       <c r="B1199" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>Babson College</t>
+        </is>
+      </c>
+      <c r="D1199" t="inlineStr">
+        <is>
+          <t>Co-author Influence Without Authority</t>
         </is>
       </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
         <is>
-          <t>Nick Morgan</t>
+          <t>William Ury</t>
         </is>
       </c>
       <c r="B1200" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Co-founder</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Harvard Negotiation Project</t>
+        </is>
+      </c>
+      <c r="D1200" t="inlineStr">
+        <is>
+          <t>Getting to Yes, principled negotiation</t>
         </is>
       </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
         <is>
-          <t>Fotini Iconomopoulos</t>
+          <t>Brian Ahearn</t>
         </is>
       </c>
       <c r="B1201" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Author &amp; Coach</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Influence PEOPLE</t>
+        </is>
+      </c>
+      <c r="D1201" t="inlineStr">
+        <is>
+          <t>Cialdini-certified influence trainer</t>
         </is>
       </c>
     </row>
     <row r="1202">
       <c r="A1202" t="inlineStr">
         <is>
-          <t>Terri Trespicio</t>
+          <t>Simon Lancaster</t>
         </is>
       </c>
       <c r="B1202" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Speechwriter &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D1202" t="inlineStr">
+        <is>
+          <t>Connect!, language of persuasion</t>
         </is>
       </c>
     </row>
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
-          <t>Jayson Gaignard</t>
+          <t>Heidi Grant</t>
         </is>
       </c>
       <c r="B1203" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Social Psychologist</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D1203" t="inlineStr">
+        <is>
+          <t>Reinforcements, motivation research</t>
         </is>
       </c>
     </row>
     <row r="1204">
       <c r="A1204" t="inlineStr">
         <is>
-          <t>Francesca Gino</t>
+          <t>Niro Sivanathan</t>
         </is>
       </c>
       <c r="B1204" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>London Business School</t>
+        </is>
+      </c>
+      <c r="D1204" t="inlineStr">
+        <is>
+          <t>Dilution effect, persuasion research</t>
         </is>
       </c>
     </row>
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t>Nir Eyal</t>
+          <t>Megan Reitz</t>
         </is>
       </c>
       <c r="B1205" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Hult Ashridge</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>Speak Up, speaking truth to power</t>
         </is>
       </c>
     </row>
     <row r="1206">
       <c r="A1206" t="inlineStr">
         <is>
-          <t>Heather Hansen</t>
+          <t>David Bradford</t>
         </is>
       </c>
       <c r="B1206" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Stanford GSB</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>Co-author Influence Without Authority</t>
         </is>
       </c>
     </row>
     <row r="1207">
       <c r="A1207" t="inlineStr">
         <is>
-          <t>Jordan Harbinger</t>
+          <t>Julie Battilana</t>
         </is>
       </c>
       <c r="B1207" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Harvard</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>Power for All, organizational influence</t>
         </is>
       </c>
     </row>
     <row r="1208">
       <c r="A1208" t="inlineStr">
         <is>
-          <t>Michael Pantalon</t>
+          <t>Nick Morgan</t>
         </is>
       </c>
       <c r="B1208" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>CEO &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Public Words</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>Communication coaching, presence</t>
         </is>
       </c>
     </row>
     <row r="1209">
       <c r="A1209" t="inlineStr">
         <is>
-          <t>G. Richard Shell</t>
+          <t>Sarah Danielle</t>
         </is>
       </c>
       <c r="B1209" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Creator</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>TikTok influence without authority content</t>
         </is>
       </c>
     </row>
     <row r="1210">
       <c r="A1210" t="inlineStr">
         <is>
-          <t>Deepak Malhotra</t>
+          <t>Caroline Goyder</t>
         </is>
       </c>
       <c r="B1210" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Author &amp; Speaking Coach</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Author of 'Gravitas'</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>TEDx 11M+ views on speaking with gravitas</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1210" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1210" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="K1210" t="inlineStr">
+        <is>
+          <t>@CarolineGoyder</t>
+        </is>
+      </c>
+      <c r="L1210" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1210" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O1210" t="inlineStr">
+        <is>
+          <t>Caroline Goyder</t>
+        </is>
+      </c>
+      <c r="P1210" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1210" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1211">
       <c r="A1211" t="inlineStr">
         <is>
-          <t>William Ury</t>
+          <t>Joel Garfinkle</t>
         </is>
       </c>
       <c r="B1211" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Garfinkle Executive Coaching</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>Amazon #1 bestseller 'Executive Presence'</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>JoelGarfinkle</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="H1211" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1211" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K1211" t="inlineStr">
+        <is>
+          <t>@joelgarfinkle</t>
+        </is>
+      </c>
+      <c r="L1211" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1211" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O1211" t="inlineStr">
+        <is>
+          <t>Joel Garfinkle</t>
+        </is>
+      </c>
+      <c r="P1211" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1211" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1212">
       <c r="A1212" t="inlineStr">
         <is>
-          <t>Linda Babcock</t>
+          <t>Muriel Maignan Wilkins</t>
         </is>
       </c>
       <c r="B1212" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>C-Suite Advisor &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Paravis Partners</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>HBR Coaching Real Leaders host</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1212" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1212" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="K1212" t="inlineStr">
+        <is>
+          <t>@MurielWilkins</t>
+        </is>
+      </c>
+      <c r="L1212" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1212" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1212" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1212" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1213">
       <c r="A1213" t="inlineStr">
         <is>
-          <t>Roger Fisher</t>
+          <t>Crystal Lim-Lange</t>
         </is>
       </c>
       <c r="B1213" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>CEO &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Forest Wolf</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>320K+ followers; Deep Human author</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>@crystallimlange</t>
+        </is>
+      </c>
+      <c r="H1213" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I1213" t="inlineStr">
+        <is>
+          <t>@crystallimlange</t>
+        </is>
+      </c>
+      <c r="J1213" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1213" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="M1213" t="inlineStr">
+        <is>
+          <t>@crystallimlange</t>
+        </is>
+      </c>
+      <c r="N1213" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P1213" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1213" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1214">
       <c r="A1214" t="inlineStr">
         <is>
-          <t>Stuart Diamond</t>
+          <t>Scott Johnston</t>
         </is>
       </c>
       <c r="B1214" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Gravitas Coach</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>ScottJohnston.net</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>Consistently Compelling Method creator</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>@1ScottJohnston</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>@coach_scott_johnston</t>
+        </is>
+      </c>
+      <c r="H1214" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="J1214" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1214" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1214" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O1214" t="inlineStr">
+        <is>
+          <t>Scott Johnston</t>
+        </is>
+      </c>
+      <c r="P1214" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1214" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1215">
       <c r="A1215" t="inlineStr">
         <is>
-          <t>Daniel Shapiro</t>
+          <t>Kara Ronin</t>
         </is>
       </c>
       <c r="B1215" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Leadership Coach</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Executive Impressions</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>275K+ YouTube subs; Udemy bestseller</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1215" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1215" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1215" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1215" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1215" t="inlineStr">
+        <is>
+          <t>Executive Impressions</t>
+        </is>
+      </c>
+      <c r="P1215" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="R1215" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1216">
       <c r="A1216" t="inlineStr">
         <is>
-          <t>Todd Davis</t>
+          <t>Sandra Zimmer</t>
         </is>
       </c>
       <c r="B1216" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Presence &amp; Speaking Coach</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Self-Expression Center</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>Pioneer in transforming stage fright since 1976</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="H1216" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1216" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1216" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1216" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1216" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1216" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1217">
       <c r="A1217" t="inlineStr">
         <is>
-          <t>Meredith Fineman</t>
+          <t>Belle Linda Halpern</t>
         </is>
       </c>
       <c r="B1217" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Leadership Presence Expert</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>The Ariel Group</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>Co-author 'Leadership Presence'</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1217" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1218">
       <c r="A1218" t="inlineStr">
         <is>
-          <t>John Baldoni</t>
+          <t>Kathy Lubar</t>
         </is>
       </c>
       <c r="B1218" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Leadership Presence Expert</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>The Ariel Group</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>Co-author 'Leadership Presence'</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1218" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1219">
       <c r="A1219" t="inlineStr">
         <is>
-          <t>Debra Benton</t>
+          <t>Janice Tomich</t>
         </is>
       </c>
       <c r="B1219" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Executive Speaking Coach</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Calculated Presentations</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>EP specialist for women leaders</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1219" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1219" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1220">
       <c r="A1220" t="inlineStr">
         <is>
-          <t>Michelle Tillis Lederman</t>
+          <t>Amy Eliza Wong</t>
         </is>
       </c>
       <c r="B1220" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Presence &amp; Communication Coach</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Always On Purpose</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>ICF-certified EP coach</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1220" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1220" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1220" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1220" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1220" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1220" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1221">
       <c r="A1221" t="inlineStr">
         <is>
-          <t>Mark Goulston</t>
+          <t>Amy Su</t>
         </is>
       </c>
       <c r="B1221" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Paravis Partners</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>Co-author 'Own the Room'</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1221" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1221" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1221" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1221" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1221" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1221" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1222">
       <c r="A1222" t="inlineStr">
         <is>
-          <t>Judith Humphrey</t>
+          <t>Benjamin Zander</t>
         </is>
       </c>
       <c r="B1222" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Conductor &amp; Speaker</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Boston Philharmonic Orchestra</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>TED legend; Art of Possibility author</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1222" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1222" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1222" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1222" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1222" t="inlineStr">
+        <is>
+          <t>Benjamin Zander</t>
+        </is>
+      </c>
+      <c r="P1222" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1222" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1223">
       <c r="A1223" t="inlineStr">
         <is>
-          <t>Bob Cialdini</t>
+          <t>Tiffany Pham</t>
         </is>
       </c>
       <c r="B1223" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>CEO &amp; Founder</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>Mogul</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>Forbes 30 Under 30; presence &amp; influence</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1223" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1223" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K1223" t="inlineStr">
+        <is>
+          <t>@taborfrompham</t>
+        </is>
+      </c>
+      <c r="L1223" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M1223" t="inlineStr">
+        <is>
+          <t>@taborfrompham</t>
+        </is>
+      </c>
+      <c r="N1223" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P1223" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1223" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1224">
       <c r="A1224" t="inlineStr">
         <is>
-          <t>Jay Conger</t>
+          <t>Ethan Evans</t>
         </is>
       </c>
       <c r="B1224" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Former VP Amazon</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Executive Coaching</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>23 years Amazon; executive presence advice</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K1224" t="inlineStr">
+        <is>
+          <t>@EthanEvansVP</t>
+        </is>
+      </c>
+      <c r="L1224" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M1224" t="inlineStr">
+        <is>
+          <t>@ethanevans</t>
+        </is>
+      </c>
+      <c r="N1224" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1224" t="inlineStr">
+        <is>
+          <t>Ethan Evans</t>
+        </is>
+      </c>
+      <c r="P1224" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1224" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1225">
       <c r="A1225" t="inlineStr">
         <is>
-          <t>Tanya Menon</t>
+          <t>Mimi Nicklin</t>
         </is>
       </c>
       <c r="B1225" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Empathy Advocate &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Empathy Everywhere</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>Bestselling author on empathetic presence</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1225" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1225" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="M1225" t="inlineStr">
+        <is>
+          <t>@miminicklin</t>
+        </is>
+      </c>
+      <c r="N1225" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1225" t="inlineStr">
+        <is>
+          <t>Mimi Nicklin</t>
+        </is>
+      </c>
+      <c r="P1225" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1225" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t>Deborah Gruenfeld</t>
+          <t>Pamela Meyer</t>
         </is>
       </c>
       <c r="B1226" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Agility Expert &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>The Agility Shift</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>Author of 'The Agility Shift' and 'Staying in the Game'</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P1226" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1226" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1227">
       <c r="A1227" t="inlineStr">
         <is>
-          <t>Brian Uzzi</t>
+          <t>Linda Holbeche</t>
         </is>
       </c>
       <c r="B1227" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>HR &amp; OD Expert</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Author &amp; Professor</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>Author of 'The Agile Organization'; former CIPD Director</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1227" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1227" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1227" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t>Simon Lancaster</t>
+          <t>Aaron De Smet</t>
         </is>
       </c>
       <c r="B1228" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Senior Partner</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>Leads McKinsey org agility research; Deliberate Calm co-author</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K1228" t="inlineStr">
+        <is>
+          <t>@AaronDeSmet</t>
+        </is>
+      </c>
+      <c r="L1228" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N1228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1228" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1228" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1229">
       <c r="A1229" t="inlineStr">
         <is>
-          <t>Charisma on Command</t>
+          <t>Jeff Sutherland</t>
         </is>
       </c>
       <c r="B1229" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Co-Creator of Scrum</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Scrum Inc.</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>Co-authored the Agile Manifesto; revolutionised project mgmt</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1229" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1229" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="K1229" t="inlineStr">
+        <is>
+          <t>@jeffsutherland</t>
+        </is>
+      </c>
+      <c r="L1229" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N1229" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1229" t="inlineStr">
+        <is>
+          <t>Scrum Inc.</t>
+        </is>
+      </c>
+      <c r="P1229" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="R1229" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1230">
       <c r="A1230" t="inlineStr">
         <is>
-          <t>Noah Zandan</t>
+          <t>Barry O'Reilly</t>
         </is>
       </c>
       <c r="B1230" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Author &amp; Entrepreneur</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Nobody Studios</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>Bestselling author of 'Unlearn'; Singularity University faculty</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="K1230" t="inlineStr">
+        <is>
+          <t>@BarryOReilly</t>
+        </is>
+      </c>
+      <c r="L1230" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N1230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1230" t="inlineStr">
+        <is>
+          <t>Barry O'Reilly</t>
+        </is>
+      </c>
+      <c r="P1230" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1230" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1231">
       <c r="A1231" t="inlineStr">
         <is>
-          <t>Chris Anderson</t>
+          <t>Nigel Thurlow</t>
         </is>
       </c>
       <c r="B1231" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Flow &amp; Agile Expert</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>The Flow Consortium</t>
+        </is>
+      </c>
+      <c r="D1231" t="inlineStr">
+        <is>
+          <t>Forbes top 10 author; trained 9,500+ in agile worldwide</t>
+        </is>
+      </c>
+      <c r="F1231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1231" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1231" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1231" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1231" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="O1231" t="inlineStr">
+        <is>
+          <t>Nigel Thurlow</t>
+        </is>
+      </c>
+      <c r="P1231" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1231" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1232">
       <c r="A1232" t="inlineStr">
         <is>
-          <t>David McRaney</t>
+          <t>Giles Lindsay</t>
         </is>
       </c>
       <c r="B1232" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Technology Executive</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>Agile Delta Consulting</t>
+        </is>
+      </c>
+      <c r="D1232" t="inlineStr">
+        <is>
+          <t>Author of 'The Adaptive Leader'; CIO/CTO recognised globally</t>
+        </is>
+      </c>
+      <c r="F1232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P1232" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1232" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1233">
       <c r="A1233" t="inlineStr">
         <is>
-          <t>Julian Treasure</t>
+          <t>Scott Graffius</t>
         </is>
       </c>
       <c r="B1233" t="inlineStr">
         <is>
-          <t>Influence Without Authority</t>
+          <t>Agile Consultant &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>Exceptional Agility</t>
+        </is>
+      </c>
+      <c r="D1233" t="inlineStr">
+        <is>
+          <t>Multi-award-winning author; 89 conferences in 25 countries</t>
+        </is>
+      </c>
+      <c r="F1233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1233" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1233" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1233" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1234">
       <c r="A1234" t="inlineStr">
         <is>
-          <t>Caroline Goyder</t>
+          <t>Christopher Worley</t>
         </is>
       </c>
       <c r="B1234" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Research Scientist</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>USC/Pepperdine</t>
+        </is>
+      </c>
+      <c r="D1234" t="inlineStr">
+        <is>
+          <t>Author of 'The Agility Factor'; agile sustainability pioneer</t>
+        </is>
+      </c>
+      <c r="F1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1234" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1234" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1235">
       <c r="A1235" t="inlineStr">
         <is>
-          <t>Olivia Fox Cabane</t>
+          <t>David Anderson</t>
         </is>
       </c>
       <c r="B1235" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Kanban Pioneer</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Kanban University</t>
+        </is>
+      </c>
+      <c r="D1235" t="inlineStr">
+        <is>
+          <t>30+ years at IBM, Motorola, Microsoft; enterprise agility</t>
+        </is>
+      </c>
+      <c r="F1235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1235" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1235" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L1235" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="O1235" t="inlineStr">
+        <is>
+          <t>Kanban University</t>
+        </is>
+      </c>
+      <c r="P1235" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1235" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1236">
       <c r="A1236" t="inlineStr">
         <is>
-          <t>Belle Linda Halpern</t>
+          <t>Bill Joiner</t>
         </is>
       </c>
       <c r="B1236" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Executive Coach &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>ChangeWise</t>
+        </is>
+      </c>
+      <c r="D1236" t="inlineStr">
+        <is>
+          <t>Co-author 'Leadership Agility: Five Levels of Mastery'</t>
+        </is>
+      </c>
+      <c r="F1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1236" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1237">
       <c r="A1237" t="inlineStr">
         <is>
-          <t>Diane Craig</t>
+          <t>Stanley McChrystal</t>
         </is>
       </c>
       <c r="B1237" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Retired General &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>McChrystal Group</t>
+        </is>
+      </c>
+      <c r="D1237" t="inlineStr">
+        <is>
+          <t>Author of 'Team of Teams'; military-to-business agility</t>
+        </is>
+      </c>
+      <c r="F1237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="K1237" t="inlineStr">
+        <is>
+          <t>@StanMcChrystal</t>
+        </is>
+      </c>
+      <c r="L1237" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N1237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1237" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="R1237" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1238">
       <c r="A1238" t="inlineStr">
         <is>
-          <t>Kristi Hedges</t>
+          <t>Peter Merel</t>
         </is>
       </c>
       <c r="B1238" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Founder &amp; Author</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>XSCALE Alliance</t>
+        </is>
+      </c>
+      <c r="D1238" t="inlineStr">
+        <is>
+          <t>Author of 'The Agile Way'; 40+ years shaping agile</t>
+        </is>
+      </c>
+      <c r="F1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1238" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1238" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1239">
       <c r="A1239" t="inlineStr">
         <is>
-          <t>Carol Kinsey Goman</t>
+          <t>Jeff Lawrence</t>
         </is>
       </c>
       <c r="B1239" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Adaptive Leadership Expert</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Org Agility Advisors</t>
+        </is>
+      </c>
+      <c r="D1239" t="inlineStr">
+        <is>
+          <t>Taught at Harvard, Oxford; systemic thinking specialist</t>
+        </is>
+      </c>
+      <c r="F1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="N1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1239" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1240">
       <c r="A1240" t="inlineStr">
         <is>
-          <t>Muriel Maignan Wilkins</t>
+          <t>Masa K Maeda</t>
         </is>
       </c>
       <c r="B1240" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Lean-Agile Expert</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>XSCALE/Kanban</t>
+        </is>
+      </c>
+      <c r="D1240" t="inlineStr">
+        <is>
+          <t>Pioneering Kanban method and enterprise evolution</t>
+        </is>
+      </c>
+      <c r="F1240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1240" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="J1240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1240" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="P1240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1240" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1241">
       <c r="A1241" t="inlineStr">
         <is>
-          <t>Lauren Sergy</t>
+          <t>Karl Smith</t>
         </is>
       </c>
       <c r="B1241" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>Agile Thought Leader</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Lean-Agile Community</t>
+        </is>
+      </c>
+      <c r="D1241" t="inlineStr">
+        <is>
+          <t>Active content creator on lean-agile practices</t>
+        </is>
+      </c>
+      <c r="F1241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="H1241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J1241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L1241" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="N1241" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="P1241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="R1241" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
         </is>
       </c>
     </row>
     <row r="1242">
       <c r="A1242" t="inlineStr">
         <is>
-          <t>Beverly Howard</t>
+          <t>Joseph Grenny</t>
         </is>
       </c>
       <c r="B1242" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>@josephgrenny</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1242" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1243">
       <c r="A1243" t="inlineStr">
         <is>
-          <t>Michael Gervais</t>
+          <t>Ryan Dunlap</t>
         </is>
       </c>
       <c r="B1243" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>@conflictish</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D1243" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1244">
       <c r="A1244" t="inlineStr">
         <is>
-          <t>Tasha Eurich</t>
+          <t>Kerry Patterson</t>
         </is>
       </c>
       <c r="B1244" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>@kerrypatterso</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1244" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1245">
       <c r="A1245" t="inlineStr">
         <is>
-          <t>Victoria Labalme</t>
-        </is>
-      </c>
-      <c r="B1245" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
+          <t>Al Switzler</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr"/>
+      <c r="C1245" t="inlineStr"/>
+      <c r="D1245" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1246">
       <c r="A1246" t="inlineStr">
         <is>
-          <t>Scott Edinger</t>
-        </is>
-      </c>
-      <c r="B1246" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
+          <t>Judy Ringer</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr"/>
+      <c r="C1246" t="inlineStr"/>
+      <c r="D1246" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1247">
       <c r="A1247" t="inlineStr">
         <is>
-          <t>Susan David</t>
+          <t>Fred Kofman</t>
         </is>
       </c>
       <c r="B1247" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>@fredkofman</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1247" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1248">
       <c r="A1248" t="inlineStr">
         <is>
-          <t>Tara Mohr</t>
+          <t>Susan Scott</t>
         </is>
       </c>
       <c r="B1248" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
+          <t>@fierceinc</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1248" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
     <row r="1249">
       <c r="A1249" t="inlineStr">
         <is>
-          <t>Vernice Armour</t>
+          <t>Karin Hurt</t>
         </is>
       </c>
       <c r="B1249" t="inlineStr">
         <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1250">
-      <c r="A1250" t="inlineStr">
-        <is>
-          <t>Peter Guber</t>
-        </is>
-      </c>
-      <c r="B1250" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1251">
-      <c r="A1251" t="inlineStr">
-        <is>
-          <t>John Neffinger</t>
-        </is>
-      </c>
-      <c r="B1251" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1252">
-      <c r="A1252" t="inlineStr">
-        <is>
-          <t>Vanessa Patrick</t>
-        </is>
-      </c>
-      <c r="B1252" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1253">
-      <c r="A1253" t="inlineStr">
-        <is>
-          <t>Ron Heifetz</t>
-        </is>
-      </c>
-      <c r="B1253" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1254">
-      <c r="A1254" t="inlineStr">
-        <is>
-          <t>Roberta Matuson</t>
-        </is>
-      </c>
-      <c r="B1254" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1255">
-      <c r="A1255" t="inlineStr">
-        <is>
-          <t>Jim Collins</t>
-        </is>
-      </c>
-      <c r="B1255" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1256">
-      <c r="A1256" t="inlineStr">
-        <is>
-          <t>Connson Locke</t>
-        </is>
-      </c>
-      <c r="B1256" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1257">
-      <c r="A1257" t="inlineStr">
-        <is>
-          <t>Joseph Grenny</t>
-        </is>
-      </c>
-      <c r="B1257" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1258">
-      <c r="A1258" t="inlineStr">
-        <is>
-          <t>Heidi Grant</t>
-        </is>
-      </c>
-      <c r="B1258" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1259">
-      <c r="A1259" t="inlineStr">
-        <is>
-          <t>Les Brown</t>
-        </is>
-      </c>
-      <c r="B1259" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1260">
-      <c r="A1260" t="inlineStr">
-        <is>
-          <t>Tom Bilyeu</t>
-        </is>
-      </c>
-      <c r="B1260" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1261">
-      <c r="A1261" t="inlineStr">
-        <is>
-          <t>Dan Pink</t>
-        </is>
-      </c>
-      <c r="B1261" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1262">
-      <c r="A1262" t="inlineStr">
-        <is>
-          <t>Patrice Washington</t>
-        </is>
-      </c>
-      <c r="B1262" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1263">
-      <c r="A1263" t="inlineStr">
-        <is>
-          <t>Chris Do</t>
-        </is>
-      </c>
-      <c r="B1263" t="inlineStr">
-        <is>
-          <t>Leadership Presence</t>
-        </is>
-      </c>
-    </row>
-    <row r="1264">
-      <c r="A1264" t="inlineStr">
-        <is>
-          <t>Aaron De Smet</t>
-        </is>
-      </c>
-      <c r="B1264" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1265">
-      <c r="A1265" t="inlineStr">
-        <is>
-          <t>Carol Dweck</t>
-        </is>
-      </c>
-      <c r="B1265" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1266">
-      <c r="A1266" t="inlineStr">
-        <is>
-          <t>Ray Dalio</t>
-        </is>
-      </c>
-      <c r="B1266" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1267">
-      <c r="A1267" t="inlineStr">
-        <is>
-          <t>Reed Hastings</t>
-        </is>
-      </c>
-      <c r="B1267" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1268">
-      <c r="A1268" t="inlineStr">
-        <is>
-          <t>Jez Humble</t>
-        </is>
-      </c>
-      <c r="B1268" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1269">
-      <c r="A1269" t="inlineStr">
-        <is>
-          <t>Jurgen Appelo</t>
-        </is>
-      </c>
-      <c r="B1269" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1270">
-      <c r="A1270" t="inlineStr">
-        <is>
-          <t>Mike Cottmeyer</t>
-        </is>
-      </c>
-      <c r="B1270" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1271">
-      <c r="A1271" t="inlineStr">
-        <is>
-          <t>Karen Martin</t>
-        </is>
-      </c>
-      <c r="B1271" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1272">
-      <c r="A1272" t="inlineStr">
-        <is>
-          <t>Mike Rother</t>
-        </is>
-      </c>
-      <c r="B1272" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1273">
-      <c r="A1273" t="inlineStr">
-        <is>
-          <t>David Marquet</t>
-        </is>
-      </c>
-      <c r="B1273" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1274">
-      <c r="A1274" t="inlineStr">
-        <is>
-          <t>Frederic Laloux</t>
-        </is>
-      </c>
-      <c r="B1274" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1275">
-      <c r="A1275" t="inlineStr">
-        <is>
-          <t>David Snowden</t>
-        </is>
-      </c>
-      <c r="B1275" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1276">
-      <c r="A1276" t="inlineStr">
-        <is>
-          <t>Tim Ferriss</t>
-        </is>
-      </c>
-      <c r="B1276" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1277">
-      <c r="A1277" t="inlineStr">
-        <is>
-          <t>Cal Newport</t>
-        </is>
-      </c>
-      <c r="B1277" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1278">
-      <c r="A1278" t="inlineStr">
-        <is>
-          <t>James Clear</t>
-        </is>
-      </c>
-      <c r="B1278" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1279">
-      <c r="A1279" t="inlineStr">
-        <is>
-          <t>Eric Ries</t>
-        </is>
-      </c>
-      <c r="B1279" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1280">
-      <c r="A1280" t="inlineStr">
-        <is>
-          <t>Steve Blank</t>
-        </is>
-      </c>
-      <c r="B1280" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1281">
-      <c r="A1281" t="inlineStr">
-        <is>
-          <t>Naval Ravikant</t>
-        </is>
-      </c>
-      <c r="B1281" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1282">
-      <c r="A1282" t="inlineStr">
-        <is>
-          <t>David Goggins</t>
-        </is>
-      </c>
-      <c r="B1282" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1283">
-      <c r="A1283" t="inlineStr">
-        <is>
-          <t>Stanley McChrystal</t>
-        </is>
-      </c>
-      <c r="B1283" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1284">
-      <c r="A1284" t="inlineStr">
-        <is>
-          <t>Gary Hamel</t>
-        </is>
-      </c>
-      <c r="B1284" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1285">
-      <c r="A1285" t="inlineStr">
-        <is>
-          <t>Charlene Li</t>
-        </is>
-      </c>
-      <c r="B1285" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1286">
-      <c r="A1286" t="inlineStr">
-        <is>
-          <t>Margaret Heffernan</t>
-        </is>
-      </c>
-      <c r="B1286" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1287">
-      <c r="A1287" t="inlineStr">
-        <is>
-          <t>Darrell Rigby</t>
-        </is>
-      </c>
-      <c r="B1287" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1288">
-      <c r="A1288" t="inlineStr">
-        <is>
-          <t>George Westerman</t>
-        </is>
-      </c>
-      <c r="B1288" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1289">
-      <c r="A1289" t="inlineStr">
-        <is>
-          <t>Tamara Erickson</t>
-        </is>
-      </c>
-      <c r="B1289" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1290">
-      <c r="A1290" t="inlineStr">
-        <is>
-          <t>Jeff Bezos</t>
-        </is>
-      </c>
-      <c r="B1290" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1291">
-      <c r="A1291" t="inlineStr">
-        <is>
-          <t>Henrik Kniberg</t>
-        </is>
-      </c>
-      <c r="B1291" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1292">
-      <c r="A1292" t="inlineStr">
-        <is>
-          <t>Marty Cagan</t>
-        </is>
-      </c>
-      <c r="B1292" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1293">
-      <c r="A1293" t="inlineStr">
-        <is>
-          <t>Gene Kim</t>
-        </is>
-      </c>
-      <c r="B1293" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1294">
-      <c r="A1294" t="inlineStr">
-        <is>
-          <t>Jeff Sutherland</t>
-        </is>
-      </c>
-      <c r="B1294" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1295">
-      <c r="A1295" t="inlineStr">
-        <is>
-          <t>Simon Wardley</t>
-        </is>
-      </c>
-      <c r="B1295" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1296">
-      <c r="A1296" t="inlineStr">
-        <is>
-          <t>Nicole Forsgren</t>
-        </is>
-      </c>
-      <c r="B1296" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1297">
-      <c r="A1297" t="inlineStr">
-        <is>
-          <t>Marc Benioff</t>
-        </is>
-      </c>
-      <c r="B1297" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1298">
-      <c r="A1298" t="inlineStr">
-        <is>
-          <t>Sundar Pichai</t>
-        </is>
-      </c>
-      <c r="B1298" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1299">
-      <c r="A1299" t="inlineStr">
-        <is>
-          <t>Dean Leffingwell</t>
-        </is>
-      </c>
-      <c r="B1299" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
-        </is>
-      </c>
-    </row>
-    <row r="1300">
-      <c r="A1300" t="inlineStr">
-        <is>
-          <t>Martin Fowler</t>
-        </is>
-      </c>
-      <c r="B1300" t="inlineStr">
-        <is>
-          <t>Organizational Agility</t>
+          <t>@letsgrowleader</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1249" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
         </is>
       </c>
     </row>
@@ -64365,7 +65587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -65717,6 +66939,66 @@
       <c r="D68" t="inlineStr">
         <is>
           <t>coaching-for-performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Influence Without Authority</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>23</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>influence-without-authority</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Leadership Presence</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>27</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>leadership-presence</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Organizational Agility</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>16</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>organizational-agility</t>
         </is>
       </c>
     </row>
@@ -65732,7 +67014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H547"/>
+  <dimension ref="A1:H555"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -85046,23 +86328,31 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>69c580337c3be86dbd857b04</t>
+          <t>60370296a73c5c70fa70c977</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>2026-04-10T21:15:00Z</t>
+          <t>69c58cbc20f76613b72d3c98</t>
         </is>
       </c>
       <c r="E524" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F524" t="inlineStr">
-        <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+      <c r="H524" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="525">
@@ -85078,23 +86368,31 @@
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>69c5803520f76613b72cff26</t>
+          <t>69bb7e247be9f8b1716f91c7</t>
         </is>
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>2026-04-11T05:01:00Z</t>
+          <t>69c58c4e20f76613b72d3a2e</t>
         </is>
       </c>
       <c r="E525" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F525" t="inlineStr">
-        <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+      <c r="H525" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="526">
@@ -85105,28 +86403,36 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>Threads</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>69c5805d7c3be86dbd857b98</t>
+          <t>69bb7e7b7be9f8b1716f927a</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>2026-04-10T16:01:00Z</t>
+          <t>69c58cef20f76613b72d3d89</t>
         </is>
       </c>
       <c r="E526" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F526" t="inlineStr">
         <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H526" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="527">
@@ -85137,28 +86443,36 @@
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>X/Twitter</t>
+          <t>Threads</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>69c5805e20f76613b72cffd7</t>
+          <t>69bb7ee47be9f8b1716f9388</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>2026-04-10T23:01:00Z</t>
+          <t>69c58cbe7c3be86dbd85b98f</t>
         </is>
       </c>
       <c r="E527" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F527" t="inlineStr">
-        <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+      <c r="H527" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="528">
@@ -85169,28 +86483,36 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>X/Twitter</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>69c5806a7c3be86dbd857bd5</t>
+          <t>69bb7fdc7be9f8b1716f9570</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>2026-04-11T01:01:00Z</t>
+          <t>69c58c697c3be86dbd85b742</t>
         </is>
       </c>
       <c r="E528" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G528" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F528" t="inlineStr">
-        <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+      <c r="H528" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="529">
@@ -85201,28 +86523,36 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>Bluesky</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>69c5806b7c3be86dbd857c0f</t>
+          <t>69bb7eff7be9f8b1716f93c9</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>2026-04-11T00:01:00Z</t>
+          <t>69c58d187c3be86dbd85baac</t>
         </is>
       </c>
       <c r="E529" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F529" t="inlineStr">
         <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="G529" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H529" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="530">
@@ -85233,28 +86563,36 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Google Business</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>69c5807520f76613b72d0030</t>
+          <t>69bb7f1d7be9f8b1716f9409</t>
         </is>
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>2026-04-14T02:00:00Z</t>
+          <t>69c58cd720f76613b72d3d21</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>customScheduled</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F530" t="inlineStr">
         <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G530" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H530" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="531">
@@ -85265,28 +86603,36 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Bluesky</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>69c580797c3be86dbd857ce0</t>
+          <t>69c08393af47dacb694508b8</t>
         </is>
       </c>
       <c r="D531" t="inlineStr">
         <is>
-          <t>2026-04-27T23:00:00Z</t>
+          <t>69c58cd87c3be86dbd85ba19</t>
         </is>
       </c>
       <c r="E531" t="inlineStr">
         <is>
-          <t>customScheduled</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F531" t="inlineStr">
         <is>
-          <t>2026-03-27 04:53</t>
-        </is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G531" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H531" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="532">
@@ -85302,23 +86648,31 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>69c582da20f76613b72d1500</t>
+          <t>60370296a73c5c70fa70c977</t>
         </is>
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>2026-04-11T00:02:00Z</t>
+          <t>69c5a24f20f76613b72db6d6</t>
         </is>
       </c>
       <c r="E532" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F532" t="inlineStr">
+        <is>
+          <t>2026-04-11T13:30:00Z</t>
+        </is>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F532" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+      <c r="H532" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="533">
@@ -85334,23 +86688,31 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>69c582db7c3be86dbd85948d</t>
+          <t>69bb7e247be9f8b1716f91c7</t>
         </is>
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>2026-04-11T08:02:00Z</t>
+          <t>69c5a25b7c3be86dbd863775</t>
         </is>
       </c>
       <c r="E533" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F533" t="inlineStr">
+        <is>
+          <t>2026-04-11T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F533" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+      <c r="H533" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="534">
@@ -85361,28 +86723,36 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>Threads</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>69c582f420f76613b72d1572</t>
+          <t>69bb7e7b7be9f8b1716f927a</t>
         </is>
       </c>
       <c r="D534" t="inlineStr">
         <is>
-          <t>2026-04-10T19:02:00Z</t>
+          <t>69c5a25c20f76613b72db745</t>
         </is>
       </c>
       <c r="E534" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F534" t="inlineStr">
         <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+          <t>2026-06-19T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H534" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="535">
@@ -85393,28 +86763,36 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>X/Twitter</t>
+          <t>Threads</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>69c582f57c3be86dbd8594e5</t>
+          <t>69bb7ee47be9f8b1716f9388</t>
         </is>
       </c>
       <c r="D535" t="inlineStr">
         <is>
-          <t>2026-04-11T02:02:00Z</t>
+          <t>69c5a2677c3be86dbd8637e0</t>
         </is>
       </c>
       <c r="E535" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F535" t="inlineStr">
+        <is>
+          <t>2026-04-11T07:01:00Z</t>
+        </is>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F535" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+      <c r="H535" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="536">
@@ -85425,28 +86803,36 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>X/Twitter</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>69c582f620f76613b72d1598</t>
+          <t>69bb7fdc7be9f8b1716f9570</t>
         </is>
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>2026-04-11T04:02:00Z</t>
+          <t>69c5a27020f76613b72db782</t>
         </is>
       </c>
       <c r="E536" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F536" t="inlineStr">
+        <is>
+          <t>2026-04-11T15:12:00Z</t>
+        </is>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F536" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+      <c r="H536" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="537">
@@ -85457,28 +86843,36 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>Bluesky</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>69c582f720f76613b72d15be</t>
+          <t>69bb7eff7be9f8b1716f93c9</t>
         </is>
       </c>
       <c r="D537" t="inlineStr">
         <is>
-          <t>2026-04-11T03:02:00Z</t>
+          <t>69c5a2767c3be86dbd86384d</t>
         </is>
       </c>
       <c r="E537" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+          <t>2026-06-10T23:00:00Z</t>
+        </is>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H537" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="538">
@@ -85489,28 +86883,36 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Google Business</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>69c583027c3be86dbd85950b</t>
+          <t>69bb7f1d7be9f8b1716f9409</t>
         </is>
       </c>
       <c r="D538" t="inlineStr">
         <is>
-          <t>2026-04-21T02:00:00Z</t>
+          <t>69c5a27b20f76613b72db7f4</t>
         </is>
       </c>
       <c r="E538" t="inlineStr">
         <is>
-          <t>customScheduled</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F538" t="inlineStr">
         <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+          <t>2026-04-11T16:01:00Z</t>
+        </is>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H538" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="539">
@@ -85521,28 +86923,36 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Bluesky</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>69c583067c3be86dbd859531</t>
+          <t>69c08393af47dacb694508b8</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
         <is>
-          <t>2026-05-04T23:00:00Z</t>
+          <t>69c5a27f7c3be86dbd863874</t>
         </is>
       </c>
       <c r="E539" t="inlineStr">
         <is>
-          <t>customScheduled</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F539" t="inlineStr">
         <is>
-          <t>2026-03-27 05:04</t>
-        </is>
+          <t>2026-04-11T13:02:00Z</t>
+        </is>
+      </c>
+      <c r="G539" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H539" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="540">
@@ -85558,23 +86968,31 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>69c584c520f76613b72d20df</t>
+          <t>60370296a73c5c70fa70c977</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
         <is>
-          <t>2026-04-11T01:01:00Z</t>
+          <t>69c5a422084613e3f1e6da7b</t>
         </is>
       </c>
       <c r="E540" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F540" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F540" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+      <c r="H540" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="541">
@@ -85590,23 +87008,31 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>69c584c77c3be86dbd859f1f</t>
+          <t>69bb7e247be9f8b1716f91c7</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">
         <is>
-          <t>2026-04-11T09:01:00Z</t>
+          <t>69c5a425084613e3f1e6daeb</t>
         </is>
       </c>
       <c r="E541" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F541" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F541" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+      <c r="H541" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="542">
@@ -85617,28 +87043,36 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Threads</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>69c584de20f76613b72d21c0</t>
+          <t>69bb7e7b7be9f8b1716f927a</t>
         </is>
       </c>
       <c r="D542" t="inlineStr">
         <is>
-          <t>2026-04-10T19:45:00Z</t>
+          <t>69c5a428084613e3f1e6db10</t>
         </is>
       </c>
       <c r="E542" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F542" t="inlineStr">
         <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H542" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="543">
@@ -85649,28 +87083,36 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>X/Twitter</t>
+          <t>Threads</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>69c584df7c3be86dbd859f79</t>
+          <t>69bb7ee47be9f8b1716f9388</t>
         </is>
       </c>
       <c r="D543" t="inlineStr">
         <is>
-          <t>2026-04-11T03:01:00Z</t>
+          <t>69c5a432d05e1e11aeea3a65</t>
         </is>
       </c>
       <c r="E543" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F543" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F543" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+      <c r="H543" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="544">
@@ -85681,28 +87123,36 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Google Business</t>
+          <t>X/Twitter</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>69c584e020f76613b72d21e6</t>
+          <t>69bb7fdc7be9f8b1716f9570</t>
         </is>
       </c>
       <c r="D544" t="inlineStr">
         <is>
-          <t>2026-04-11T05:01:00Z</t>
+          <t>69c5a43c084613e3f1e6dbf5</t>
         </is>
       </c>
       <c r="E544" t="inlineStr">
         <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F544" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
           <t>addToQueue</t>
         </is>
       </c>
-      <c r="F544" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+      <c r="H544" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="545">
@@ -85713,28 +87163,36 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>Bluesky</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>69c584e17c3be86dbd859f9f</t>
+          <t>69bb7eff7be9f8b1716f93c9</t>
         </is>
       </c>
       <c r="D545" t="inlineStr">
         <is>
-          <t>2026-04-11T03:45:00Z</t>
+          <t>69c5a441d05e1e11aeea3b1d</t>
         </is>
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>addToQueue</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>customScheduled</t>
+        </is>
+      </c>
+      <c r="H545" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="546">
@@ -85745,28 +87203,36 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Google Business</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>69c584ec7c3be86dbd859fea</t>
+          <t>69bb7f1d7be9f8b1716f9409</t>
         </is>
       </c>
       <c r="D546" t="inlineStr">
         <is>
-          <t>2026-04-28T02:00:00Z</t>
+          <t>69c5a447d05e1e11aeea3b57</t>
         </is>
       </c>
       <c r="E546" t="inlineStr">
         <is>
-          <t>customScheduled</t>
+          <t>scheduled</t>
         </is>
       </c>
       <c r="F546" t="inlineStr">
         <is>
-          <t>2026-03-27 05:12</t>
-        </is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H546" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="547">
@@ -85777,27 +87243,251 @@
       </c>
       <c r="B547" t="inlineStr">
         <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>69c08393af47dacb694508b8</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>69c5a449084613e3f1e6dc49</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+      <c r="F547" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>addToQueue</t>
+        </is>
+      </c>
+      <c r="H547" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>69c5a799084613e3f1e6ec78</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>69c5a7a9084613e3f1e6ecae</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>69c5a7abd05e1e11aeea4ff6</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>69c5a98f084613e3f1e6f422</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>69c5a992084613e3f1e6f448</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>69c5a996d05e1e11aeea578a</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>69c5a9a0d05e1e11aeea5852</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="C547" t="inlineStr">
-        <is>
-          <t>69c584f07c3be86dbd85a010</t>
-        </is>
-      </c>
-      <c r="D547" t="inlineStr">
-        <is>
-          <t>2026-05-11T23:00:00Z</t>
-        </is>
-      </c>
-      <c r="E547" t="inlineStr">
-        <is>
-          <t>customScheduled</t>
-        </is>
-      </c>
-      <c r="F547" t="inlineStr">
-        <is>
-          <t>2026-03-27 05:12</t>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>69c5a9a3d05e1e11aeea5881</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>scheduled</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update handle-database: Employee Engagement complete (Topic 4/4) — all 4 topics done
</commit_message>
<xml_diff>
--- a/Cowork-Data/multi-platform-social-post/handle-database.xlsx
+++ b/Cowork-Data/multi-platform-social-post/handle-database.xlsx
@@ -2243,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1249"/>
+  <dimension ref="A1:Y1265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -65487,8 +65487,6 @@
           <t>Al Switzler</t>
         </is>
       </c>
-      <c r="B1245" t="inlineStr"/>
-      <c r="C1245" t="inlineStr"/>
       <c r="D1245" t="inlineStr">
         <is>
           <t>Difficult Conversations</t>
@@ -65501,8 +65499,6 @@
           <t>Judy Ringer</t>
         </is>
       </c>
-      <c r="B1246" t="inlineStr"/>
-      <c r="C1246" t="inlineStr"/>
       <c r="D1246" t="inlineStr">
         <is>
           <t>Difficult Conversations</t>
@@ -65572,6 +65568,350 @@
       <c r="D1249" t="inlineStr">
         <is>
           <t>Difficult Conversations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>Marcus Buckingham</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>@mbuckingham</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1250" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>Marcus Buckingham</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>@marcusbuckingham</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D1251" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>Jim Harter</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>@jimharter</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1252" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>Kevin Kruse</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>@kevinkruse</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1253" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>David Zinger</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>@davezinger</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1254" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>Laszlo Bock</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>@laszlobock</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1255" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>Chester Elton</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>@chesterelton</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1256" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>Adrian Gostick</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>@adriangostick</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1257" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>Jacob Morgan</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>@jacobmorgan</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1258" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>Josh Bersin</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>@josh_bersin</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1259" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>Dan Pink</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>@DanielPink</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1260" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>Arianna Huffington</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>@araborescottnn</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1261" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>Michael Bungay Stanier</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>@BungayStanier</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1262" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>Patty McCord</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>@patty_mccord</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1263" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>Shawn Achor</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>@shawnachor</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="D1264" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>Bob Nelson</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr"/>
+      <c r="C1265" t="inlineStr"/>
+      <c r="D1265" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
         </is>
       </c>
     </row>
@@ -67014,7 +67354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H555"/>
+  <dimension ref="A1:H563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -87491,6 +87831,222 @@
         </is>
       </c>
     </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>69c5ab84084613e3f1e6f8ec</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>69c5ab8bd05e1e11aeea5cde</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>69c5ab8d084613e3f1e6f95d</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Threads</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>69c5aba0d05e1e11aeea5d3a</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>X/Twitter</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>69c5aba3084613e3f1e6f9aa</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Bluesky</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>69c5aba6d05e1e11aeea5d60</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Google Business</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>69c5abb0084613e3f1e6f9dd</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Employee Engagement</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>69c5abb3d05e1e11aeea5dbf</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>scheduled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>